<commit_message>
Update TS2#90 Note via Tab3
</commit_message>
<xml_diff>
--- a/TS2_note.xlsx
+++ b/TS2_note.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>NOTE</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NOTICE</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +454,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -466,6 +476,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -483,6 +498,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -500,6 +520,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -517,6 +542,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -534,6 +564,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -551,6 +586,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -568,6 +608,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -585,6 +630,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -602,6 +652,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -619,6 +674,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -636,6 +696,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -653,6 +718,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -670,6 +740,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -687,6 +762,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -704,6 +784,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -721,6 +806,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -738,6 +828,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -755,6 +850,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -772,6 +872,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -789,6 +894,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -806,6 +916,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -823,6 +938,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -840,6 +960,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -857,6 +982,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -874,6 +1004,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -891,6 +1026,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -908,6 +1048,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -925,6 +1070,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -942,6 +1092,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -959,6 +1114,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -976,6 +1136,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -993,6 +1158,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1010,6 +1180,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1027,6 +1202,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1044,6 +1224,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1061,6 +1246,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1078,6 +1268,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1095,6 +1290,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1112,6 +1312,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1129,6 +1334,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1146,6 +1356,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1163,6 +1378,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1180,6 +1400,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1197,6 +1422,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1214,6 +1444,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1231,6 +1466,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1248,6 +1488,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1265,6 +1510,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1282,6 +1532,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1299,6 +1554,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1316,6 +1576,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1333,6 +1598,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1350,6 +1620,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1367,6 +1642,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1384,6 +1664,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1401,6 +1686,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1418,6 +1708,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1435,6 +1730,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1452,6 +1752,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1469,6 +1774,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1486,6 +1796,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1503,6 +1818,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1520,6 +1840,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1537,6 +1862,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1554,6 +1884,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1571,6 +1906,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1588,6 +1928,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1605,6 +1950,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1622,6 +1972,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1639,6 +1994,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1656,6 +2016,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1673,6 +2038,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1690,6 +2060,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1707,6 +2082,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1724,6 +2104,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1741,6 +2126,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1758,6 +2148,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1775,6 +2170,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1792,6 +2192,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1809,6 +2214,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1826,6 +2236,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1843,6 +2258,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1860,6 +2280,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1877,6 +2302,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1894,6 +2324,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1911,6 +2346,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1928,6 +2368,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1945,6 +2390,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1962,6 +2412,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1979,6 +2434,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1996,6 +2456,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2013,6 +2478,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2030,6 +2500,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2047,6 +2522,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2064,6 +2544,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2081,6 +2566,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2098,6 +2588,11 @@
           <t>無資料</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2111,6 +2606,11 @@
         </is>
       </c>
       <c r="C100" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
         <is>
           <t>無資料</t>
         </is>

</xml_diff>

<commit_message>
Update TS2#71 Note via Tab3
</commit_message>
<xml_diff>
--- a/TS2_note.xlsx
+++ b/TS2_note.xlsx
@@ -1993,12 +1993,13 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>無資料</t>
+          <t>09/24 09:23 TS2#71  FT(P) pass
+HS_COLD on going</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>無資料</t>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update TS2#79 Note via Tab3
</commit_message>
<xml_diff>
--- a/TS2_note.xlsx
+++ b/TS2_note.xlsx
@@ -2171,12 +2171,13 @@
       <c r="C80" t="inlineStr">
         <is>
           <t>9/23 09:30 發現有光纖插反+斷掉需更換
-9/23 15:06  換fiber中</t>
+9/23 15:06  換fiber中
+9/24 04:36 FT(p) pass</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bulk update NOTICE for 3 systems via Streamlit
</commit_message>
<xml_diff>
--- a/TS2_note.xlsx
+++ b/TS2_note.xlsx
@@ -2308,7 +2308,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>